<commit_message>
Added new RDF data schemes and visual schemes for economy-table134-137, fixed XLSX spreadsheet for economy-table134
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table134.xlsx
+++ b/sources/table_normalization/xlsx/economy-table134.xlsx
@@ -656,8 +656,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="#0.000"/>
-    <numFmt numFmtId="169" formatCode="#0.0"/>
+    <numFmt numFmtId="164" formatCode="#0.000"/>
+    <numFmt numFmtId="165" formatCode="#0.0"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -711,7 +711,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -732,17 +732,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -750,20 +756,18 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1068,59 +1072,59 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="14"/>
     </row>
     <row r="2" spans="1:23">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="14"/>
     </row>
     <row r="3" spans="1:23">
       <c r="A3" s="2" t="s">
@@ -1152,39 +1156,39 @@
       <c r="W3" s="4"/>
     </row>
     <row r="4" spans="1:23" s="1" customFormat="1" ht="31">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14" t="s">
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="S4" s="14"/>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
+      <c r="S4" s="15"/>
+      <c r="T4" s="15"/>
+      <c r="U4" s="15"/>
+      <c r="V4" s="15"/>
+      <c r="W4" s="15"/>
     </row>
     <row r="5" spans="1:23" ht="28">
       <c r="A5" s="4"/>
@@ -1332,22 +1336,22 @@
       <c r="Q7" s="8">
         <v>312.33199999999999</v>
       </c>
-      <c r="R7" s="11">
+      <c r="R7" s="10">
         <v>3.5</v>
       </c>
-      <c r="S7" s="11">
+      <c r="S7" s="10">
         <v>1.3</v>
       </c>
-      <c r="T7" s="11">
+      <c r="T7" s="10">
         <v>0.6</v>
       </c>
-      <c r="U7" s="11">
+      <c r="U7" s="10">
         <v>3.2</v>
       </c>
-      <c r="V7" s="11">
+      <c r="V7" s="10">
         <v>1.2</v>
       </c>
-      <c r="W7" s="11">
+      <c r="W7" s="10">
         <v>0.6</v>
       </c>
     </row>
@@ -1359,11 +1363,15 @@
         <v>24</v>
       </c>
     </row>
+    <row r="10" spans="1:23">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+    </row>
     <row r="11" spans="1:23">
-      <c r="A11" s="6">
+      <c r="A11" s="16">
         <v>1</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="19" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="7" t="s">
@@ -1411,30 +1419,30 @@
       <c r="Q11" s="8">
         <v>321.74099999999999</v>
       </c>
-      <c r="R11" s="11">
+      <c r="R11" s="10">
         <v>3.4</v>
       </c>
-      <c r="S11" s="11">
+      <c r="S11" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="T11" s="11">
+      <c r="T11" s="10">
         <v>0.7</v>
       </c>
-      <c r="U11" s="11">
+      <c r="U11" s="10">
         <v>2.4</v>
       </c>
-      <c r="V11" s="11">
+      <c r="V11" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="W11" s="11">
+      <c r="W11" s="10">
         <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="1:23">
-      <c r="A12" s="6">
+      <c r="A12" s="16">
         <v>2</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="20" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="7" t="s">
@@ -1482,30 +1490,30 @@
       <c r="Q12" s="8">
         <v>325.50299999999999</v>
       </c>
-      <c r="R12" s="11">
+      <c r="R12" s="10">
         <v>3.5</v>
       </c>
-      <c r="S12" s="11">
+      <c r="S12" s="10">
         <v>0.9</v>
       </c>
-      <c r="T12" s="11">
+      <c r="T12" s="10">
         <v>0.5</v>
       </c>
-      <c r="U12" s="11">
+      <c r="U12" s="10">
         <v>2.9</v>
       </c>
-      <c r="V12" s="11">
+      <c r="V12" s="10">
         <v>1.2</v>
       </c>
-      <c r="W12" s="11">
+      <c r="W12" s="10">
         <v>0.4</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="16.5">
-      <c r="A13" s="6">
+      <c r="A13" s="16">
         <v>2</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="20" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="7" t="s">
@@ -1553,30 +1561,30 @@
       <c r="Q13" s="8">
         <v>189.446</v>
       </c>
-      <c r="R13" s="11">
+      <c r="R13" s="10">
         <v>3.2</v>
       </c>
-      <c r="S13" s="11">
+      <c r="S13" s="10">
         <v>1.4</v>
       </c>
-      <c r="T13" s="11">
+      <c r="T13" s="10">
         <v>0.9</v>
       </c>
-      <c r="U13" s="11">
+      <c r="U13" s="10">
         <v>1.9</v>
       </c>
-      <c r="V13" s="11">
+      <c r="V13" s="10">
         <v>1</v>
       </c>
-      <c r="W13" s="11">
+      <c r="W13" s="10">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="16.5">
-      <c r="A14" s="6">
+      <c r="A14" s="16">
         <v>2</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="20" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="7" t="s">
@@ -1624,30 +1632,30 @@
       <c r="Q14" s="8">
         <v>122.807</v>
       </c>
-      <c r="R14" s="11">
+      <c r="R14" s="10">
         <v>3.1</v>
       </c>
-      <c r="S14" s="11">
+      <c r="S14" s="10">
         <v>1.3</v>
       </c>
-      <c r="T14" s="11">
+      <c r="T14" s="10">
         <v>1</v>
       </c>
-      <c r="U14" s="11">
+      <c r="U14" s="10">
         <v>2.1</v>
       </c>
-      <c r="V14" s="11">
+      <c r="V14" s="10">
         <v>0.9</v>
       </c>
-      <c r="W14" s="11">
+      <c r="W14" s="10">
         <v>0.4</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="16.5">
-      <c r="A15" s="6">
+      <c r="A15" s="16">
         <v>2</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="20" t="s">
         <v>29</v>
       </c>
       <c r="C15" s="7" t="s">
@@ -1695,30 +1703,34 @@
       <c r="Q15" s="8">
         <v>123.601</v>
       </c>
-      <c r="R15" s="11">
+      <c r="R15" s="10">
         <v>3.5</v>
       </c>
-      <c r="S15" s="11">
+      <c r="S15" s="10">
         <v>1</v>
       </c>
-      <c r="T15" s="11">
+      <c r="T15" s="10">
         <v>0.6</v>
       </c>
-      <c r="U15" s="11">
+      <c r="U15" s="10">
         <v>2.6</v>
       </c>
-      <c r="V15" s="11">
+      <c r="V15" s="10">
         <v>1.2</v>
       </c>
-      <c r="W15" s="11">
+      <c r="W15" s="10">
         <v>0.5</v>
       </c>
     </row>
+    <row r="16" spans="1:23">
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+    </row>
     <row r="17" spans="1:23">
-      <c r="A17" s="6">
+      <c r="A17" s="16">
         <v>1</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="19" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="7" t="s">
@@ -1766,30 +1778,30 @@
       <c r="Q17" s="8">
         <v>288.30099999999999</v>
       </c>
-      <c r="R17" s="11">
+      <c r="R17" s="10">
         <v>2.8</v>
       </c>
-      <c r="S17" s="11">
+      <c r="S17" s="10">
         <v>1.3</v>
       </c>
-      <c r="T17" s="11">
+      <c r="T17" s="10">
         <v>0.7</v>
       </c>
-      <c r="U17" s="11">
+      <c r="U17" s="10">
         <v>2.8</v>
       </c>
-      <c r="V17" s="11">
+      <c r="V17" s="10">
         <v>0.9</v>
       </c>
-      <c r="W17" s="11">
+      <c r="W17" s="10">
         <v>0.6</v>
       </c>
     </row>
     <row r="18" spans="1:23">
-      <c r="A18" s="6">
+      <c r="A18" s="16">
         <v>2</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="20" t="s">
         <v>31</v>
       </c>
       <c r="C18" s="7" t="s">
@@ -1837,30 +1849,30 @@
       <c r="Q18" s="8">
         <v>288.10399999999998</v>
       </c>
-      <c r="R18" s="11">
+      <c r="R18" s="10">
         <v>3.3</v>
       </c>
-      <c r="S18" s="11">
+      <c r="S18" s="10">
         <v>1.4</v>
       </c>
-      <c r="T18" s="11">
+      <c r="T18" s="10">
         <v>0.8</v>
       </c>
-      <c r="U18" s="11">
+      <c r="U18" s="10">
         <v>3.2</v>
       </c>
-      <c r="V18" s="11">
+      <c r="V18" s="10">
         <v>1</v>
       </c>
-      <c r="W18" s="11">
+      <c r="W18" s="10">
         <v>0.6</v>
       </c>
     </row>
     <row r="19" spans="1:23" ht="16.5">
-      <c r="A19" s="6">
+      <c r="A19" s="16">
         <v>2</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="20" t="s">
         <v>32</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -1908,30 +1920,30 @@
       <c r="Q19" s="8">
         <v>184.667</v>
       </c>
-      <c r="R19" s="11">
+      <c r="R19" s="10">
         <v>2.6</v>
       </c>
-      <c r="S19" s="11">
+      <c r="S19" s="10">
         <v>1.2</v>
       </c>
-      <c r="T19" s="11">
+      <c r="T19" s="10">
         <v>0.6</v>
       </c>
-      <c r="U19" s="11">
+      <c r="U19" s="10">
         <v>2.5</v>
       </c>
-      <c r="V19" s="11">
+      <c r="V19" s="10">
         <v>0.8</v>
       </c>
-      <c r="W19" s="11">
+      <c r="W19" s="10">
         <v>0.5</v>
       </c>
     </row>
     <row r="20" spans="1:23" ht="16.5">
-      <c r="A20" s="6">
+      <c r="A20" s="16">
         <v>2</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C20" s="7" t="s">
@@ -1979,30 +1991,30 @@
       <c r="Q20" s="8">
         <v>124.812</v>
       </c>
-      <c r="R20" s="11">
+      <c r="R20" s="10">
         <v>2.6</v>
       </c>
-      <c r="S20" s="11">
+      <c r="S20" s="10">
         <v>1.2</v>
       </c>
-      <c r="T20" s="11">
+      <c r="T20" s="10">
         <v>0.7</v>
       </c>
-      <c r="U20" s="11">
+      <c r="U20" s="10">
         <v>2.6</v>
       </c>
-      <c r="V20" s="11">
+      <c r="V20" s="10">
         <v>0.9</v>
       </c>
-      <c r="W20" s="11">
+      <c r="W20" s="10">
         <v>0.5</v>
       </c>
     </row>
     <row r="21" spans="1:23" ht="16.5">
-      <c r="A21" s="6">
+      <c r="A21" s="16">
         <v>2</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="20" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="7" t="s">
@@ -2050,30 +2062,34 @@
       <c r="Q21" s="8">
         <v>125.62</v>
       </c>
-      <c r="R21" s="11">
+      <c r="R21" s="10">
         <v>3.4</v>
       </c>
-      <c r="S21" s="11">
+      <c r="S21" s="10">
         <v>1.4</v>
       </c>
-      <c r="T21" s="11">
+      <c r="T21" s="10">
         <v>0.6</v>
       </c>
-      <c r="U21" s="11">
+      <c r="U21" s="10">
         <v>3</v>
       </c>
-      <c r="V21" s="11">
+      <c r="V21" s="10">
         <v>0.9</v>
       </c>
-      <c r="W21" s="11">
+      <c r="W21" s="10">
         <v>0.8</v>
       </c>
     </row>
+    <row r="22" spans="1:23">
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+    </row>
     <row r="23" spans="1:23">
-      <c r="A23" s="6">
+      <c r="A23" s="16">
         <v>1</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="19" t="s">
         <v>35</v>
       </c>
       <c r="C23" s="7" t="s">
@@ -2121,30 +2137,30 @@
       <c r="Q23" s="8">
         <v>304.49</v>
       </c>
-      <c r="R23" s="11">
+      <c r="R23" s="10">
         <v>3.8</v>
       </c>
-      <c r="S23" s="11">
+      <c r="S23" s="10">
         <v>1.4</v>
       </c>
-      <c r="T23" s="11">
+      <c r="T23" s="10">
         <v>0.4</v>
       </c>
-      <c r="U23" s="11">
+      <c r="U23" s="10">
         <v>3.7</v>
       </c>
-      <c r="V23" s="11">
+      <c r="V23" s="10">
         <v>1.5</v>
       </c>
-      <c r="W23" s="11">
+      <c r="W23" s="10">
         <v>0.9</v>
       </c>
     </row>
     <row r="24" spans="1:23">
-      <c r="A24" s="6">
+      <c r="A24" s="16">
         <v>2</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C24" s="7" t="s">
@@ -2192,30 +2208,30 @@
       <c r="Q24" s="8">
         <v>310.72300000000001</v>
       </c>
-      <c r="R24" s="11">
+      <c r="R24" s="10">
         <v>3.9</v>
       </c>
-      <c r="S24" s="11">
+      <c r="S24" s="10">
         <v>1.3</v>
       </c>
-      <c r="T24" s="11">
+      <c r="T24" s="10">
         <v>0.4</v>
       </c>
-      <c r="U24" s="11">
+      <c r="U24" s="10">
         <v>4.0999999999999996</v>
       </c>
-      <c r="V24" s="11">
+      <c r="V24" s="10">
         <v>1.2</v>
       </c>
-      <c r="W24" s="11">
+      <c r="W24" s="10">
         <v>0.9</v>
       </c>
     </row>
     <row r="25" spans="1:23" ht="16.5">
-      <c r="A25" s="6">
+      <c r="A25" s="16">
         <v>2</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="20" t="s">
         <v>37</v>
       </c>
       <c r="C25" s="7" t="s">
@@ -2263,30 +2279,30 @@
       <c r="Q25" s="8">
         <v>192.26400000000001</v>
       </c>
-      <c r="R25" s="11">
+      <c r="R25" s="10">
         <v>3.7</v>
       </c>
-      <c r="S25" s="11">
+      <c r="S25" s="10">
         <v>1.4</v>
       </c>
-      <c r="T25" s="11">
+      <c r="T25" s="10">
         <v>0.5</v>
       </c>
-      <c r="U25" s="11">
+      <c r="U25" s="10">
         <v>3.5</v>
       </c>
-      <c r="V25" s="11">
+      <c r="V25" s="10">
         <v>1.6</v>
       </c>
-      <c r="W25" s="11">
+      <c r="W25" s="10">
         <v>0.9</v>
       </c>
     </row>
     <row r="26" spans="1:23" ht="16.5">
-      <c r="A26" s="6">
+      <c r="A26" s="16">
         <v>2</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="20" t="s">
         <v>38</v>
       </c>
       <c r="C26" s="7" t="s">
@@ -2334,30 +2350,30 @@
       <c r="Q26" s="8">
         <v>129.33799999999999</v>
       </c>
-      <c r="R26" s="11">
+      <c r="R26" s="10">
         <v>3.9</v>
       </c>
-      <c r="S26" s="11">
+      <c r="S26" s="10">
         <v>1.4</v>
       </c>
-      <c r="T26" s="11">
+      <c r="T26" s="10">
         <v>0.4</v>
       </c>
-      <c r="U26" s="11">
+      <c r="U26" s="10">
         <v>3.9</v>
       </c>
-      <c r="V26" s="11">
+      <c r="V26" s="10">
         <v>1.4</v>
       </c>
-      <c r="W26" s="11">
+      <c r="W26" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:23" ht="16.5">
-      <c r="A27" s="6">
+      <c r="A27" s="16">
         <v>2</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="20" t="s">
         <v>39</v>
       </c>
       <c r="C27" s="7" t="s">
@@ -2405,30 +2421,30 @@
       <c r="Q27" s="8">
         <v>126.131</v>
       </c>
-      <c r="R27" s="11">
+      <c r="R27" s="10">
         <v>4</v>
       </c>
-      <c r="S27" s="11">
+      <c r="S27" s="10">
         <v>1.6</v>
       </c>
-      <c r="T27" s="11">
+      <c r="T27" s="10">
         <v>0.7</v>
       </c>
-      <c r="U27" s="11">
+      <c r="U27" s="10">
         <v>3.5</v>
       </c>
-      <c r="V27" s="11">
+      <c r="V27" s="10">
         <v>1.7</v>
       </c>
-      <c r="W27" s="11">
+      <c r="W27" s="10">
         <v>0.9</v>
       </c>
     </row>
     <row r="28" spans="1:23" ht="16.5">
-      <c r="A28" s="6">
+      <c r="A28" s="16">
         <v>2</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="20" t="s">
         <v>40</v>
       </c>
       <c r="C28" s="7" t="s">
@@ -2476,30 +2492,34 @@
       <c r="Q28" s="8">
         <v>125.31399999999999</v>
       </c>
-      <c r="R28" s="11">
+      <c r="R28" s="10">
         <v>3.6</v>
       </c>
-      <c r="S28" s="11">
+      <c r="S28" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="T28" s="11">
+      <c r="T28" s="10">
         <v>0.3</v>
       </c>
-      <c r="U28" s="11">
+      <c r="U28" s="10">
         <v>3.5</v>
       </c>
-      <c r="V28" s="11">
+      <c r="V28" s="10">
         <v>1.5</v>
       </c>
-      <c r="W28" s="11">
+      <c r="W28" s="10">
         <v>0.8</v>
       </c>
     </row>
+    <row r="29" spans="1:23">
+      <c r="A29" s="18"/>
+      <c r="B29" s="18"/>
+    </row>
     <row r="30" spans="1:23">
-      <c r="A30" s="6">
+      <c r="A30" s="16">
         <v>1</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="19" t="s">
         <v>41</v>
       </c>
       <c r="C30" s="7" t="s">
@@ -2547,30 +2567,30 @@
       <c r="Q30" s="8">
         <v>332.202</v>
       </c>
-      <c r="R30" s="11">
+      <c r="R30" s="10">
         <v>3.6</v>
       </c>
-      <c r="S30" s="11">
+      <c r="S30" s="10">
         <v>1.3</v>
       </c>
-      <c r="T30" s="11">
+      <c r="T30" s="10">
         <v>0.9</v>
       </c>
-      <c r="U30" s="11">
+      <c r="U30" s="10">
         <v>3.2</v>
       </c>
-      <c r="V30" s="11">
+      <c r="V30" s="10">
         <v>1</v>
       </c>
-      <c r="W30" s="11">
+      <c r="W30" s="10">
         <v>0.4</v>
       </c>
     </row>
     <row r="31" spans="1:23">
-      <c r="A31" s="6">
+      <c r="A31" s="16">
         <v>2</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="20" t="s">
         <v>42</v>
       </c>
       <c r="C31" s="7" t="s">
@@ -2618,30 +2638,30 @@
       <c r="Q31" s="8">
         <v>341.29899999999998</v>
       </c>
-      <c r="R31" s="11">
+      <c r="R31" s="10">
         <v>3.6</v>
       </c>
-      <c r="S31" s="11">
+      <c r="S31" s="10">
         <v>1.2</v>
       </c>
-      <c r="T31" s="11">
+      <c r="T31" s="10">
         <v>0.6</v>
       </c>
-      <c r="U31" s="11">
+      <c r="U31" s="10">
         <v>3.2</v>
       </c>
-      <c r="V31" s="11">
+      <c r="V31" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="W31" s="11">
+      <c r="W31" s="10">
         <v>0.6</v>
       </c>
     </row>
     <row r="32" spans="1:23" ht="16.5">
-      <c r="A32" s="6">
+      <c r="A32" s="16">
         <v>2</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="20" t="s">
         <v>43</v>
       </c>
       <c r="C32" s="7" t="s">
@@ -2689,30 +2709,30 @@
       <c r="Q32" s="8">
         <v>194.047</v>
       </c>
-      <c r="R32" s="11">
+      <c r="R32" s="10">
         <v>3.6</v>
       </c>
-      <c r="S32" s="11">
+      <c r="S32" s="10">
         <v>1.3</v>
       </c>
-      <c r="T32" s="11">
+      <c r="T32" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="U32" s="11">
+      <c r="U32" s="10">
         <v>3.2</v>
       </c>
-      <c r="V32" s="11">
+      <c r="V32" s="10">
         <v>0.9</v>
       </c>
-      <c r="W32" s="11">
+      <c r="W32" s="10">
         <v>0.2</v>
       </c>
     </row>
     <row r="33" spans="1:23" ht="16.5">
-      <c r="A33" s="6">
+      <c r="A33" s="16">
         <v>2</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="20" t="s">
         <v>44</v>
       </c>
       <c r="C33" s="7" t="s">
@@ -2760,30 +2780,30 @@
       <c r="Q33" s="8">
         <v>131.17599999999999</v>
       </c>
-      <c r="R33" s="11">
+      <c r="R33" s="10">
         <v>2.5</v>
       </c>
-      <c r="S33" s="11">
+      <c r="S33" s="10">
         <v>1</v>
       </c>
-      <c r="T33" s="11">
+      <c r="T33" s="10">
         <v>0.9</v>
       </c>
-      <c r="U33" s="11">
+      <c r="U33" s="10">
         <v>2.5</v>
       </c>
-      <c r="V33" s="11">
+      <c r="V33" s="10">
         <v>0.7</v>
       </c>
-      <c r="W33" s="11">
+      <c r="W33" s="10">
         <v>0.2</v>
       </c>
     </row>
     <row r="34" spans="1:23" ht="16.5">
-      <c r="A34" s="6">
+      <c r="A34" s="16">
         <v>2</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="20" t="s">
         <v>45</v>
       </c>
       <c r="C34" s="7" t="s">
@@ -2831,24 +2851,28 @@
       <c r="Q34" s="8">
         <v>128.34100000000001</v>
       </c>
-      <c r="R34" s="11">
+      <c r="R34" s="10">
         <v>4</v>
       </c>
-      <c r="S34" s="11">
+      <c r="S34" s="10">
         <v>1.3</v>
       </c>
-      <c r="T34" s="11">
+      <c r="T34" s="10">
         <v>0.9</v>
       </c>
-      <c r="U34" s="11">
+      <c r="U34" s="10">
         <v>3.5</v>
       </c>
-      <c r="V34" s="11">
+      <c r="V34" s="10">
         <v>1.2</v>
       </c>
-      <c r="W34" s="11">
+      <c r="W34" s="10">
         <v>0.5</v>
       </c>
+    </row>
+    <row r="35" spans="1:23">
+      <c r="A35" s="18"/>
+      <c r="B35" s="18"/>
     </row>
     <row r="36" spans="1:23">
       <c r="A36" s="16">
@@ -2858,11 +2882,15 @@
         <v>46</v>
       </c>
     </row>
+    <row r="37" spans="1:23">
+      <c r="A37" s="18"/>
+      <c r="B37" s="18"/>
+    </row>
     <row r="38" spans="1:23" ht="16.5">
-      <c r="A38" s="6">
+      <c r="A38" s="16">
         <v>1</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="19" t="s">
         <v>47</v>
       </c>
       <c r="C38" s="7" t="s">
@@ -2910,30 +2938,30 @@
       <c r="Q38" s="8">
         <v>287.13799999999998</v>
       </c>
-      <c r="R38" s="11">
+      <c r="R38" s="10">
         <v>3.6</v>
       </c>
-      <c r="S38" s="11">
+      <c r="S38" s="10">
         <v>1.2</v>
       </c>
-      <c r="T38" s="11">
+      <c r="T38" s="10">
         <v>0.5</v>
       </c>
-      <c r="U38" s="11">
+      <c r="U38" s="10">
         <v>3.4</v>
       </c>
-      <c r="V38" s="11">
+      <c r="V38" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="W38" s="11">
+      <c r="W38" s="10">
         <v>0.6</v>
       </c>
     </row>
     <row r="39" spans="1:23" ht="16.5">
-      <c r="A39" s="6">
+      <c r="A39" s="16">
         <v>1</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="19" t="s">
         <v>48</v>
       </c>
       <c r="C39" s="7" t="s">
@@ -2981,24 +3009,28 @@
       <c r="Q39" s="8">
         <v>190.607</v>
       </c>
-      <c r="R39" s="11">
+      <c r="R39" s="10">
         <v>3.4</v>
       </c>
-      <c r="S39" s="11">
+      <c r="S39" s="10">
         <v>1.3</v>
       </c>
-      <c r="T39" s="11">
+      <c r="T39" s="10">
         <v>0.7</v>
       </c>
-      <c r="U39" s="11">
+      <c r="U39" s="10">
         <v>3</v>
       </c>
-      <c r="V39" s="11">
+      <c r="V39" s="10">
         <v>1.2</v>
       </c>
-      <c r="W39" s="11">
+      <c r="W39" s="10">
         <v>0.6</v>
       </c>
+    </row>
+    <row r="40" spans="1:23">
+      <c r="A40" s="18"/>
+      <c r="B40" s="18"/>
     </row>
     <row r="41" spans="1:23">
       <c r="A41" s="16">
@@ -3008,6 +3040,10 @@
         <v>49</v>
       </c>
     </row>
+    <row r="42" spans="1:23">
+      <c r="A42" s="18"/>
+      <c r="B42" s="18"/>
+    </row>
     <row r="43" spans="1:23">
       <c r="A43" s="6">
         <v>1</v>
@@ -3060,22 +3096,22 @@
       <c r="Q43" s="8">
         <v>289.06900000000002</v>
       </c>
-      <c r="R43" s="11">
+      <c r="R43" s="10">
         <v>3.1</v>
       </c>
-      <c r="S43" s="11">
+      <c r="S43" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="T43" s="11">
+      <c r="T43" s="10">
         <v>0.6</v>
       </c>
-      <c r="U43" s="11">
+      <c r="U43" s="10">
         <v>3.4</v>
       </c>
-      <c r="V43" s="11">
+      <c r="V43" s="10">
         <v>1.3</v>
       </c>
-      <c r="W43" s="11">
+      <c r="W43" s="10">
         <v>0.5</v>
       </c>
     </row>
@@ -3131,22 +3167,22 @@
       <c r="Q44" s="8">
         <v>330.67099999999999</v>
       </c>
-      <c r="R44" s="11">
+      <c r="R44" s="10">
         <v>4</v>
       </c>
-      <c r="S44" s="11">
+      <c r="S44" s="10">
         <v>1.2</v>
       </c>
-      <c r="T44" s="11">
+      <c r="T44" s="10">
         <v>0.7</v>
       </c>
-      <c r="U44" s="11">
+      <c r="U44" s="10">
         <v>3.4</v>
       </c>
-      <c r="V44" s="11">
+      <c r="V44" s="10">
         <v>1.5</v>
       </c>
-      <c r="W44" s="11">
+      <c r="W44" s="10">
         <v>0.5</v>
       </c>
     </row>
@@ -3202,22 +3238,22 @@
       <c r="Q45" s="8">
         <v>329.82900000000001</v>
       </c>
-      <c r="R45" s="11">
+      <c r="R45" s="10">
         <v>3.4</v>
       </c>
-      <c r="S45" s="11">
+      <c r="S45" s="10">
         <v>0.6</v>
       </c>
-      <c r="T45" s="11">
+      <c r="T45" s="10">
         <v>0.4</v>
       </c>
-      <c r="U45" s="11">
+      <c r="U45" s="10">
         <v>2.9</v>
       </c>
-      <c r="V45" s="11">
+      <c r="V45" s="10">
         <v>1.2</v>
       </c>
-      <c r="W45" s="11">
+      <c r="W45" s="10">
         <v>0.2</v>
       </c>
     </row>
@@ -3262,10 +3298,10 @@
       <c r="R47" s="7"/>
       <c r="S47" s="7"/>
       <c r="T47" s="7"/>
-      <c r="U47" s="11">
+      <c r="U47" s="10">
         <v>3.3</v>
       </c>
-      <c r="V47" s="11">
+      <c r="V47" s="10">
         <v>1.3</v>
       </c>
       <c r="W47" s="7"/>
@@ -3311,10 +3347,10 @@
       <c r="R48" s="7"/>
       <c r="S48" s="7"/>
       <c r="T48" s="7"/>
-      <c r="U48" s="11">
+      <c r="U48" s="10">
         <v>2.6</v>
       </c>
-      <c r="V48" s="11">
+      <c r="V48" s="10">
         <v>1.7</v>
       </c>
       <c r="W48" s="7"/>
@@ -3360,10 +3396,10 @@
       <c r="R49" s="7"/>
       <c r="S49" s="7"/>
       <c r="T49" s="7"/>
-      <c r="U49" s="11">
+      <c r="U49" s="10">
         <v>2.8</v>
       </c>
-      <c r="V49" s="11">
+      <c r="V49" s="10">
         <v>0.2</v>
       </c>
       <c r="W49" s="7"/>
@@ -3409,10 +3445,10 @@
       <c r="R50" s="7"/>
       <c r="S50" s="7"/>
       <c r="T50" s="7"/>
-      <c r="U50" s="11">
+      <c r="U50" s="10">
         <v>3.5</v>
       </c>
-      <c r="V50" s="11">
+      <c r="V50" s="10">
         <v>1</v>
       </c>
       <c r="W50" s="7"/>
@@ -3458,10 +3494,10 @@
       <c r="R51" s="7"/>
       <c r="S51" s="7"/>
       <c r="T51" s="7"/>
-      <c r="U51" s="11">
+      <c r="U51" s="10">
         <v>4.9000000000000004</v>
       </c>
-      <c r="V51" s="11">
+      <c r="V51" s="10">
         <v>1.4</v>
       </c>
       <c r="W51" s="7"/>
@@ -3507,10 +3543,10 @@
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
-      <c r="U52" s="11">
+      <c r="U52" s="10">
         <v>3.4</v>
       </c>
-      <c r="V52" s="11">
+      <c r="V52" s="10">
         <v>1.6</v>
       </c>
       <c r="W52" s="7"/>
@@ -3556,10 +3592,10 @@
       <c r="R53" s="7"/>
       <c r="S53" s="7"/>
       <c r="T53" s="7"/>
-      <c r="U53" s="11">
+      <c r="U53" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="V53" s="11">
+      <c r="V53" s="10">
         <v>0.7</v>
       </c>
       <c r="W53" s="7"/>
@@ -3605,10 +3641,10 @@
       <c r="R54" s="7"/>
       <c r="S54" s="7"/>
       <c r="T54" s="7"/>
-      <c r="U54" s="11">
+      <c r="U54" s="10">
         <v>2.4</v>
       </c>
-      <c r="V54" s="11">
+      <c r="V54" s="10">
         <v>1.5</v>
       </c>
       <c r="W54" s="7"/>
@@ -3654,10 +3690,10 @@
       <c r="R55" s="7"/>
       <c r="S55" s="7"/>
       <c r="T55" s="7"/>
-      <c r="U55" s="11">
+      <c r="U55" s="10">
         <v>4.3</v>
       </c>
-      <c r="V55" s="11">
+      <c r="V55" s="10">
         <v>1.2</v>
       </c>
       <c r="W55" s="7"/>
@@ -3703,10 +3739,10 @@
       <c r="R56" s="7"/>
       <c r="S56" s="7"/>
       <c r="T56" s="7"/>
-      <c r="U56" s="11">
+      <c r="U56" s="10">
         <v>3.6</v>
       </c>
-      <c r="V56" s="11">
+      <c r="V56" s="10">
         <v>1.6</v>
       </c>
       <c r="W56" s="7"/>
@@ -3752,10 +3788,10 @@
       <c r="R57" s="7"/>
       <c r="S57" s="7"/>
       <c r="T57" s="7"/>
-      <c r="U57" s="11">
+      <c r="U57" s="10">
         <v>1.7</v>
       </c>
-      <c r="V57" s="11">
+      <c r="V57" s="10">
         <v>0.1</v>
       </c>
       <c r="W57" s="7"/>
@@ -3798,10 +3834,10 @@
       <c r="Q59" s="8">
         <v>335.59899999999999</v>
       </c>
-      <c r="R59" s="11">
+      <c r="R59" s="10">
         <v>3.3</v>
       </c>
-      <c r="S59" s="11">
+      <c r="S59" s="10">
         <v>1.5</v>
       </c>
       <c r="T59" s="7"/>
@@ -3847,10 +3883,10 @@
       <c r="Q60" s="8">
         <v>298.71899999999999</v>
       </c>
-      <c r="R60" s="11">
+      <c r="R60" s="10">
         <v>4.9000000000000004</v>
       </c>
-      <c r="S60" s="11">
+      <c r="S60" s="10">
         <v>0.9</v>
       </c>
       <c r="T60" s="7"/>
@@ -3896,10 +3932,10 @@
       <c r="Q61" s="8">
         <v>325.48500000000001</v>
       </c>
-      <c r="R61" s="11">
+      <c r="R61" s="10">
         <v>2.8</v>
       </c>
-      <c r="S61" s="11">
+      <c r="S61" s="10">
         <v>0.7</v>
       </c>
       <c r="T61" s="7"/>
@@ -3945,10 +3981,10 @@
       <c r="Q62" s="8">
         <v>297.76900000000001</v>
       </c>
-      <c r="R62" s="11">
+      <c r="R62" s="10">
         <v>2.7</v>
       </c>
-      <c r="S62" s="11">
+      <c r="S62" s="10">
         <v>0.6</v>
       </c>
       <c r="T62" s="7"/>
@@ -3994,10 +4030,10 @@
       <c r="Q63" s="8">
         <v>133.14400000000001</v>
       </c>
-      <c r="R63" s="11">
+      <c r="R63" s="10">
         <v>4.3</v>
       </c>
-      <c r="S63" s="11">
+      <c r="S63" s="10">
         <v>1.4</v>
       </c>
       <c r="T63" s="7"/>
@@ -4043,10 +4079,10 @@
       <c r="Q64" s="8">
         <v>370.858</v>
       </c>
-      <c r="R64" s="11">
+      <c r="R64" s="10">
         <v>3.6</v>
       </c>
-      <c r="S64" s="11">
+      <c r="S64" s="10">
         <v>0.8</v>
       </c>
       <c r="T64" s="7"/>
@@ -4092,10 +4128,10 @@
       <c r="Q65" s="8">
         <v>299.02999999999997</v>
       </c>
-      <c r="R65" s="11">
+      <c r="R65" s="10">
         <v>3.7</v>
       </c>
-      <c r="S65" s="11">
+      <c r="S65" s="10">
         <v>0.9</v>
       </c>
       <c r="T65" s="7"/>
@@ -4141,10 +4177,10 @@
       <c r="Q66" s="8">
         <v>338.06</v>
       </c>
-      <c r="R66" s="11">
+      <c r="R66" s="10">
         <v>4.8</v>
       </c>
-      <c r="S66" s="11">
+      <c r="S66" s="10">
         <v>1.5</v>
       </c>
       <c r="T66" s="7"/>
@@ -4190,10 +4226,10 @@
       <c r="Q67" s="8">
         <v>313.108</v>
       </c>
-      <c r="R67" s="11">
+      <c r="R67" s="10">
         <v>3.4</v>
       </c>
-      <c r="S67" s="11">
+      <c r="S67" s="10">
         <v>1</v>
       </c>
       <c r="T67" s="7"/>
@@ -4234,7 +4270,7 @@
       <c r="A69" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B69" s="15" t="s">
+      <c r="B69" s="12" t="s">
         <v>75</v>
       </c>
       <c r="C69" s="4"/>
@@ -4263,7 +4299,7 @@
       <c r="A70" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B70" s="15" t="s">
+      <c r="B70" s="12" t="s">
         <v>76</v>
       </c>
       <c r="C70" s="4"/>
@@ -4292,7 +4328,7 @@
       <c r="A71" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B71" s="15" t="s">
+      <c r="B71" s="12" t="s">
         <v>77</v>
       </c>
       <c r="C71" s="4"/>
@@ -4321,7 +4357,7 @@
       <c r="A72" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B72" s="15" t="s">
+      <c r="B72" s="12" t="s">
         <v>78</v>
       </c>
       <c r="C72" s="4"/>
@@ -4350,7 +4386,7 @@
       <c r="A73" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B73" s="15" t="s">
+      <c r="B73" s="12" t="s">
         <v>79</v>
       </c>
       <c r="C73" s="4"/>
@@ -4379,7 +4415,7 @@
       <c r="A74" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B74" s="15" t="s">
+      <c r="B74" s="12" t="s">
         <v>80</v>
       </c>
       <c r="C74" s="4"/>
@@ -4408,7 +4444,7 @@
       <c r="A75" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B75" s="15" t="s">
+      <c r="B75" s="12" t="s">
         <v>81</v>
       </c>
       <c r="C75" s="4"/>
@@ -4437,7 +4473,7 @@
       <c r="A76" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B76" s="15" t="s">
+      <c r="B76" s="12" t="s">
         <v>82</v>
       </c>
       <c r="C76" s="4"/>
@@ -4466,7 +4502,7 @@
       <c r="A77" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B77" s="15" t="s">
+      <c r="B77" s="12" t="s">
         <v>83</v>
       </c>
       <c r="C77" s="4"/>
@@ -4495,7 +4531,7 @@
       <c r="A78" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B78" s="15" t="s">
+      <c r="B78" s="12" t="s">
         <v>84</v>
       </c>
       <c r="C78" s="4"/>

</xml_diff>